<commit_message>
Update Guest Sync logic and stabilize Online Sheet view
</commit_message>
<xml_diff>
--- a/hiruom.xlsx
+++ b/hiruom.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29922"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25928"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d99f142bd70df661/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dewmo\Pictures\hiruayurvedaresort\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0D3C84E0-9499-4CA6-A3B2-1AE1C942769B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AB687B2-4AB6-428E-950D-0604B17E535C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -11434,8 +11434,13 @@
     <xf numFmtId="17" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -11448,12 +11453,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -11736,6 +11736,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AS1185"/>
   <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="41" width="4" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="23.25">
       <c r="A1" s="325">
@@ -18438,8 +18441,8 @@
       <c r="D121" s="9"/>
       <c r="E121" s="9"/>
       <c r="F121" s="9"/>
-      <c r="G121" s="328"/>
-      <c r="H121" s="329"/>
+      <c r="G121" s="331"/>
+      <c r="H121" s="339"/>
       <c r="I121" s="82" t="s">
         <v>238</v>
       </c>
@@ -31401,7 +31404,7 @@
       <c r="AP352" s="322"/>
       <c r="AQ352" s="322"/>
       <c r="AR352" s="321"/>
-      <c r="AS352" s="330"/>
+      <c r="AS352" s="335"/>
     </row>
     <row r="353" spans="1:45">
       <c r="A353" s="3" t="s">
@@ -31452,7 +31455,7 @@
       <c r="AP353" s="322"/>
       <c r="AQ353" s="322"/>
       <c r="AR353" s="139"/>
-      <c r="AS353" s="330"/>
+      <c r="AS353" s="335"/>
     </row>
     <row r="354" spans="1:45">
       <c r="A354" s="2">
@@ -31566,7 +31569,7 @@
       <c r="AP355" s="322"/>
       <c r="AQ355" s="322"/>
       <c r="AR355" s="321"/>
-      <c r="AS355" s="330"/>
+      <c r="AS355" s="335"/>
     </row>
     <row r="356" spans="1:45">
       <c r="A356" s="2">
@@ -31623,7 +31626,7 @@
       <c r="AP356" s="322"/>
       <c r="AQ356" s="322"/>
       <c r="AR356" s="321"/>
-      <c r="AS356" s="330"/>
+      <c r="AS356" s="335"/>
     </row>
     <row r="357" spans="1:45">
       <c r="A357" s="2">
@@ -31731,7 +31734,7 @@
       <c r="AP358" s="322"/>
       <c r="AQ358" s="322"/>
       <c r="AR358" s="145"/>
-      <c r="AS358" s="330"/>
+      <c r="AS358" s="335"/>
     </row>
     <row r="359" spans="1:45">
       <c r="A359" s="2">
@@ -31788,7 +31791,7 @@
       <c r="AP359" s="323"/>
       <c r="AQ359" s="323"/>
       <c r="AR359" s="321"/>
-      <c r="AS359" s="330"/>
+      <c r="AS359" s="335"/>
     </row>
     <row r="360" spans="1:45">
       <c r="A360" s="2">
@@ -31841,11 +31844,11 @@
       <c r="AL360" s="1"/>
       <c r="AM360" s="1"/>
       <c r="AN360" s="1"/>
-      <c r="AO360" s="331"/>
-      <c r="AP360" s="332"/>
+      <c r="AO360" s="336"/>
+      <c r="AP360" s="337"/>
       <c r="AQ360" s="323"/>
-      <c r="AR360" s="333"/>
-      <c r="AS360" s="330"/>
+      <c r="AR360" s="338"/>
+      <c r="AS360" s="335"/>
     </row>
     <row r="361" spans="1:45">
       <c r="A361" s="2">
@@ -31898,11 +31901,11 @@
       <c r="AL361" s="1"/>
       <c r="AM361" s="1"/>
       <c r="AN361" s="1"/>
-      <c r="AO361" s="331"/>
-      <c r="AP361" s="332"/>
+      <c r="AO361" s="336"/>
+      <c r="AP361" s="337"/>
       <c r="AQ361" s="323"/>
-      <c r="AR361" s="333"/>
-      <c r="AS361" s="330"/>
+      <c r="AR361" s="338"/>
+      <c r="AS361" s="335"/>
     </row>
     <row r="362" spans="1:45">
       <c r="A362" s="7">
@@ -35738,7 +35741,7 @@
       <c r="AR429" s="1"/>
       <c r="AS429" s="1"/>
     </row>
-    <row r="430" spans="1:45" ht="15.75">
+    <row r="430" spans="1:45">
       <c r="A430" s="2">
         <v>12</v>
       </c>
@@ -36042,7 +36045,7 @@
       <c r="AR435" s="1"/>
       <c r="AS435" s="1"/>
     </row>
-    <row r="436" spans="1:45" ht="15.75">
+    <row r="436" spans="1:45">
       <c r="A436" s="2">
         <v>15</v>
       </c>
@@ -36936,7 +36939,7 @@
       <c r="AR451" s="1"/>
       <c r="AS451" s="1"/>
     </row>
-    <row r="452" spans="1:45" ht="15.75">
+    <row r="452" spans="1:45">
       <c r="A452" s="2">
         <v>12</v>
       </c>
@@ -36987,7 +36990,7 @@
       <c r="AR452" s="1"/>
       <c r="AS452" s="1"/>
     </row>
-    <row r="453" spans="1:45" ht="15.75">
+    <row r="453" spans="1:45">
       <c r="A453" s="2">
         <v>14</v>
       </c>
@@ -37038,7 +37041,7 @@
       <c r="AR453" s="1"/>
       <c r="AS453" s="1"/>
     </row>
-    <row r="454" spans="1:45" ht="15.75">
+    <row r="454" spans="1:45">
       <c r="A454" s="21" t="s">
         <v>26</v>
       </c>
@@ -37087,7 +37090,7 @@
       <c r="AR454" s="1"/>
       <c r="AS454" s="1"/>
     </row>
-    <row r="455" spans="1:45" ht="15.75">
+    <row r="455" spans="1:45">
       <c r="A455" s="22" t="s">
         <v>27</v>
       </c>
@@ -37136,7 +37139,7 @@
       <c r="AR455" s="1"/>
       <c r="AS455" s="1"/>
     </row>
-    <row r="456" spans="1:45" ht="15.75">
+    <row r="456" spans="1:45">
       <c r="A456" s="22" t="s">
         <v>29</v>
       </c>
@@ -37185,7 +37188,7 @@
       <c r="AR456" s="1"/>
       <c r="AS456" s="1"/>
     </row>
-    <row r="457" spans="1:45" ht="15.75">
+    <row r="457" spans="1:45">
       <c r="A457" s="21" t="s">
         <v>31</v>
       </c>
@@ -37234,7 +37237,7 @@
       <c r="AR457" s="1"/>
       <c r="AS457" s="1"/>
     </row>
-    <row r="458" spans="1:45" ht="15.75">
+    <row r="458" spans="1:45">
       <c r="A458" s="2">
         <v>15</v>
       </c>
@@ -38042,7 +38045,7 @@
       <c r="AR471" s="1"/>
       <c r="AS471" s="1"/>
     </row>
-    <row r="472" spans="1:45" ht="15.75">
+    <row r="472" spans="1:45">
       <c r="A472" s="2">
         <v>11</v>
       </c>
@@ -38097,7 +38100,7 @@
       <c r="AR472" s="1"/>
       <c r="AS472" s="1"/>
     </row>
-    <row r="473" spans="1:45" ht="15.75">
+    <row r="473" spans="1:45">
       <c r="A473" s="2">
         <v>12</v>
       </c>
@@ -38152,7 +38155,7 @@
       <c r="AR473" s="1"/>
       <c r="AS473" s="1"/>
     </row>
-    <row r="474" spans="1:45" ht="15.75">
+    <row r="474" spans="1:45">
       <c r="A474" s="2">
         <v>14</v>
       </c>
@@ -38203,7 +38206,7 @@
       <c r="AR474" s="1"/>
       <c r="AS474" s="1"/>
     </row>
-    <row r="475" spans="1:45" ht="15.75">
+    <row r="475" spans="1:45">
       <c r="A475" s="21" t="s">
         <v>26</v>
       </c>
@@ -38252,7 +38255,7 @@
       <c r="AR475" s="1"/>
       <c r="AS475" s="1"/>
     </row>
-    <row r="476" spans="1:45" ht="15.75">
+    <row r="476" spans="1:45">
       <c r="A476" s="22" t="s">
         <v>27</v>
       </c>
@@ -38305,7 +38308,7 @@
       <c r="AR476" s="1"/>
       <c r="AS476" s="1"/>
     </row>
-    <row r="477" spans="1:45" ht="15.75">
+    <row r="477" spans="1:45">
       <c r="A477" s="22" t="s">
         <v>29</v>
       </c>
@@ -40160,7 +40163,7 @@
       <c r="AR509" s="1"/>
       <c r="AS509" s="1"/>
     </row>
-    <row r="510" spans="1:45" ht="15.75">
+    <row r="510" spans="1:45">
       <c r="A510" s="2">
         <v>5</v>
       </c>
@@ -40274,7 +40277,7 @@
       <c r="AR511" s="1"/>
       <c r="AS511" s="1"/>
     </row>
-    <row r="512" spans="1:45" ht="15.75">
+    <row r="512" spans="1:45">
       <c r="A512" s="2">
         <v>7</v>
       </c>
@@ -40384,7 +40387,7 @@
       <c r="AR513" s="1"/>
       <c r="AS513" s="1"/>
     </row>
-    <row r="514" spans="1:45" ht="15.75">
+    <row r="514" spans="1:45">
       <c r="A514" s="2">
         <v>10</v>
       </c>
@@ -42355,10 +42358,10 @@
       <c r="C549" s="7"/>
       <c r="D549" s="7"/>
       <c r="E549" s="7"/>
-      <c r="F549" s="334" t="s">
+      <c r="F549" s="333" t="s">
         <v>1121</v>
       </c>
-      <c r="G549" s="335"/>
+      <c r="G549" s="334"/>
       <c r="H549" s="13"/>
       <c r="I549" s="39"/>
       <c r="J549" s="13"/>
@@ -42783,7 +42786,7 @@
       <c r="AR556" s="1"/>
       <c r="AS556" s="1"/>
     </row>
-    <row r="557" spans="1:45" ht="15.75">
+    <row r="557" spans="1:45">
       <c r="A557" s="2">
         <v>10</v>
       </c>
@@ -43215,7 +43218,7 @@
       <c r="AR564" s="1"/>
       <c r="AS564" s="1"/>
     </row>
-    <row r="565" spans="1:45" ht="15.75">
+    <row r="565" spans="1:45">
       <c r="A565" s="2">
         <v>15</v>
       </c>
@@ -45002,7 +45005,7 @@
       <c r="AR595" s="1"/>
       <c r="AS595" s="1"/>
     </row>
-    <row r="596" spans="1:45" ht="15.75">
+    <row r="596" spans="1:45">
       <c r="A596" s="2">
         <v>5</v>
       </c>
@@ -45059,7 +45062,7 @@
       <c r="AR596" s="1"/>
       <c r="AS596" s="1"/>
     </row>
-    <row r="597" spans="1:45" ht="15.75">
+    <row r="597" spans="1:45">
       <c r="A597" s="2">
         <v>6</v>
       </c>
@@ -45114,7 +45117,7 @@
       <c r="AR597" s="1"/>
       <c r="AS597" s="1"/>
     </row>
-    <row r="598" spans="1:45" ht="15.75">
+    <row r="598" spans="1:45">
       <c r="A598" s="2">
         <v>7</v>
       </c>
@@ -45169,7 +45172,7 @@
       <c r="AR598" s="1"/>
       <c r="AS598" s="1"/>
     </row>
-    <row r="599" spans="1:45" ht="15.75">
+    <row r="599" spans="1:45">
       <c r="A599" s="7">
         <v>8</v>
       </c>
@@ -45499,7 +45502,7 @@
       <c r="AR604" s="1"/>
       <c r="AS604" s="1"/>
     </row>
-    <row r="605" spans="1:45" ht="15.75">
+    <row r="605" spans="1:45">
       <c r="A605" s="22" t="s">
         <v>27</v>
       </c>
@@ -45713,7 +45716,7 @@
       <c r="AR608" s="1"/>
       <c r="AS608" s="1"/>
     </row>
-    <row r="609" spans="1:45" ht="15.75">
+    <row r="609" spans="1:45">
       <c r="A609" s="2"/>
       <c r="B609" s="7"/>
       <c r="C609" s="2"/>
@@ -45766,7 +45769,7 @@
       <c r="AR609" s="1"/>
       <c r="AS609" s="1"/>
     </row>
-    <row r="610" spans="1:45" ht="15.75">
+    <row r="610" spans="1:45">
       <c r="A610" s="2"/>
       <c r="B610" s="7"/>
       <c r="C610" s="2"/>
@@ -46134,7 +46137,7 @@
       <c r="AR615" s="1"/>
       <c r="AS615" s="1"/>
     </row>
-    <row r="616" spans="1:45" ht="15.75">
+    <row r="616" spans="1:45">
       <c r="A616" s="2">
         <v>3</v>
       </c>
@@ -46246,7 +46249,7 @@
       <c r="AR617" s="1"/>
       <c r="AS617" s="1"/>
     </row>
-    <row r="618" spans="1:45" ht="15.75">
+    <row r="618" spans="1:45">
       <c r="A618" s="3" t="s">
         <v>6</v>
       </c>
@@ -46297,7 +46300,7 @@
       <c r="AR618" s="1"/>
       <c r="AS618" s="1"/>
     </row>
-    <row r="619" spans="1:45" ht="15.75">
+    <row r="619" spans="1:45">
       <c r="A619" s="2">
         <v>5</v>
       </c>
@@ -46354,7 +46357,7 @@
       <c r="AR619" s="1"/>
       <c r="AS619" s="1"/>
     </row>
-    <row r="620" spans="1:45" ht="15.75">
+    <row r="620" spans="1:45">
       <c r="A620" s="2">
         <v>6</v>
       </c>
@@ -46411,7 +46414,7 @@
       <c r="AR620" s="1"/>
       <c r="AS620" s="1"/>
     </row>
-    <row r="621" spans="1:45" ht="15.75">
+    <row r="621" spans="1:45">
       <c r="A621" s="2">
         <v>7</v>
       </c>
@@ -46466,7 +46469,7 @@
       <c r="AR621" s="1"/>
       <c r="AS621" s="1"/>
     </row>
-    <row r="622" spans="1:45" ht="15.75">
+    <row r="622" spans="1:45">
       <c r="A622" s="7">
         <v>8</v>
       </c>
@@ -46523,7 +46526,7 @@
       <c r="AR622" s="1"/>
       <c r="AS622" s="1"/>
     </row>
-    <row r="623" spans="1:45" ht="15.75">
+    <row r="623" spans="1:45">
       <c r="A623" s="2">
         <v>10</v>
       </c>
@@ -46580,7 +46583,7 @@
       <c r="AR623" s="1"/>
       <c r="AS623" s="1"/>
     </row>
-    <row r="624" spans="1:45" ht="15.75">
+    <row r="624" spans="1:45">
       <c r="A624" s="2">
         <v>11</v>
       </c>
@@ -46798,7 +46801,7 @@
       <c r="AR627" s="1"/>
       <c r="AS627" s="1"/>
     </row>
-    <row r="628" spans="1:45" ht="15.75">
+    <row r="628" spans="1:45">
       <c r="A628" s="22" t="s">
         <v>27</v>
       </c>
@@ -46855,7 +46858,7 @@
       <c r="AR628" s="1"/>
       <c r="AS628" s="1"/>
     </row>
-    <row r="629" spans="1:45" ht="15.75">
+    <row r="629" spans="1:45">
       <c r="A629" s="22" t="s">
         <v>29</v>
       </c>
@@ -47178,7 +47181,7 @@
       <c r="AR633" s="1"/>
       <c r="AS633" s="1"/>
     </row>
-    <row r="634" spans="1:45" ht="15.75">
+    <row r="634" spans="1:45">
       <c r="A634" s="3" t="s">
         <v>0</v>
       </c>
@@ -47229,7 +47232,7 @@
       <c r="AR634" s="1"/>
       <c r="AS634" s="1"/>
     </row>
-    <row r="635" spans="1:45" ht="15.75">
+    <row r="635" spans="1:45">
       <c r="A635" s="2">
         <v>1</v>
       </c>
@@ -47288,7 +47291,7 @@
       <c r="AR635" s="1"/>
       <c r="AS635" s="1"/>
     </row>
-    <row r="636" spans="1:45" ht="15.75">
+    <row r="636" spans="1:45">
       <c r="A636" s="2">
         <v>2</v>
       </c>
@@ -47563,7 +47566,7 @@
       <c r="AR640" s="1"/>
       <c r="AS640" s="1"/>
     </row>
-    <row r="641" spans="1:45" ht="15.75">
+    <row r="641" spans="1:45">
       <c r="A641" s="2">
         <v>6</v>
       </c>
@@ -47620,7 +47623,7 @@
       <c r="AR641" s="1"/>
       <c r="AS641" s="1"/>
     </row>
-    <row r="642" spans="1:45" ht="15.75">
+    <row r="642" spans="1:45">
       <c r="A642" s="2">
         <v>7</v>
       </c>
@@ -47905,7 +47908,7 @@
       <c r="AR646" s="1"/>
       <c r="AS646" s="1"/>
     </row>
-    <row r="647" spans="1:45" ht="15.75">
+    <row r="647" spans="1:45">
       <c r="A647" s="2">
         <v>14</v>
       </c>
@@ -48815,7 +48818,7 @@
       <c r="AR662" s="1"/>
       <c r="AS662" s="1"/>
     </row>
-    <row r="663" spans="1:45" ht="15.75">
+    <row r="663" spans="1:45">
       <c r="A663" s="2">
         <v>7</v>
       </c>
@@ -49041,7 +49044,7 @@
       <c r="AR666" s="1"/>
       <c r="AS666" s="1"/>
     </row>
-    <row r="667" spans="1:45" ht="15.75">
+    <row r="667" spans="1:45">
       <c r="A667" s="2">
         <v>12</v>
       </c>
@@ -49896,7 +49899,7 @@
       <c r="AR681" s="1"/>
       <c r="AS681" s="1"/>
     </row>
-    <row r="682" spans="1:45" ht="15.75">
+    <row r="682" spans="1:45">
       <c r="A682" s="2">
         <v>5</v>
       </c>
@@ -52078,7 +52081,7 @@
       <c r="AR721" s="1"/>
       <c r="AS721" s="1"/>
     </row>
-    <row r="722" spans="1:45" ht="15.75">
+    <row r="722" spans="1:45">
       <c r="A722" s="2">
         <v>4</v>
       </c>
@@ -53607,7 +53610,7 @@
       <c r="AR750" s="1"/>
       <c r="AS750" s="1"/>
     </row>
-    <row r="751" spans="1:45" ht="15.75">
+    <row r="751" spans="1:45">
       <c r="A751" s="2">
         <v>10</v>
       </c>
@@ -53660,7 +53663,7 @@
       <c r="AR751" s="1"/>
       <c r="AS751" s="1"/>
     </row>
-    <row r="752" spans="1:45" ht="15.75">
+    <row r="752" spans="1:45">
       <c r="A752" s="2">
         <v>11</v>
       </c>
@@ -53713,7 +53716,7 @@
       <c r="AR752" s="1"/>
       <c r="AS752" s="1"/>
     </row>
-    <row r="753" spans="1:45" ht="15.75">
+    <row r="753" spans="1:45">
       <c r="A753" s="2">
         <v>12</v>
       </c>
@@ -54587,7 +54590,7 @@
       <c r="AR768" s="1"/>
       <c r="AS768" s="1"/>
     </row>
-    <row r="769" spans="1:45" ht="15.75">
+    <row r="769" spans="1:45">
       <c r="A769" s="3" t="s">
         <v>6</v>
       </c>
@@ -54638,7 +54641,7 @@
       <c r="AR769" s="1"/>
       <c r="AS769" s="1"/>
     </row>
-    <row r="770" spans="1:45" ht="15.75">
+    <row r="770" spans="1:45">
       <c r="A770" s="2">
         <v>5</v>
       </c>
@@ -54978,10 +54981,10 @@
       <c r="C776" s="44"/>
       <c r="D776" s="44"/>
       <c r="E776" s="43"/>
-      <c r="F776" s="336"/>
-      <c r="G776" s="337"/>
-      <c r="H776" s="337"/>
-      <c r="I776" s="338"/>
+      <c r="F776" s="330"/>
+      <c r="G776" s="328"/>
+      <c r="H776" s="328"/>
+      <c r="I776" s="329"/>
       <c r="J776" s="2"/>
       <c r="K776" s="2"/>
       <c r="L776" s="2"/>
@@ -57518,16 +57521,16 @@
       <c r="T821" s="44"/>
       <c r="U821" s="44"/>
       <c r="V821" s="44"/>
-      <c r="W821" s="328" t="s">
+      <c r="W821" s="331" t="s">
         <v>1667</v>
       </c>
-      <c r="X821" s="339"/>
-      <c r="Y821" s="339"/>
-      <c r="Z821" s="339"/>
-      <c r="AA821" s="339"/>
-      <c r="AB821" s="339"/>
-      <c r="AC821" s="339"/>
-      <c r="AD821" s="339"/>
+      <c r="X821" s="332"/>
+      <c r="Y821" s="332"/>
+      <c r="Z821" s="332"/>
+      <c r="AA821" s="332"/>
+      <c r="AB821" s="332"/>
+      <c r="AC821" s="332"/>
+      <c r="AD821" s="332"/>
       <c r="AE821" s="81"/>
       <c r="AF821" s="2"/>
       <c r="AG821" s="2"/>
@@ -57711,7 +57714,7 @@
       <c r="AR824" s="1"/>
       <c r="AS824" s="1"/>
     </row>
-    <row r="825" spans="1:45" ht="15.75">
+    <row r="825" spans="1:45">
       <c r="A825" s="22" t="s">
         <v>27</v>
       </c>
@@ -57760,7 +57763,7 @@
       <c r="AR825" s="1"/>
       <c r="AS825" s="1"/>
     </row>
-    <row r="826" spans="1:45" ht="15.75">
+    <row r="826" spans="1:45">
       <c r="A826" s="22" t="s">
         <v>29</v>
       </c>
@@ -57811,7 +57814,7 @@
       <c r="AR826" s="1"/>
       <c r="AS826" s="1"/>
     </row>
-    <row r="827" spans="1:45" ht="15.75">
+    <row r="827" spans="1:45">
       <c r="A827" s="21" t="s">
         <v>31</v>
       </c>
@@ -59002,7 +59005,7 @@
       <c r="AR847" s="1"/>
       <c r="AS847" s="1"/>
     </row>
-    <row r="848" spans="1:45" ht="15.75">
+    <row r="848" spans="1:45">
       <c r="A848" s="22" t="s">
         <v>27</v>
       </c>
@@ -59696,7 +59699,7 @@
       <c r="AR859" s="1"/>
       <c r="AS859" s="1"/>
     </row>
-    <row r="860" spans="1:45" ht="15.75">
+    <row r="860" spans="1:45">
       <c r="A860" s="2">
         <v>3</v>
       </c>
@@ -59753,7 +59756,7 @@
       <c r="AR860" s="1"/>
       <c r="AS860" s="1"/>
     </row>
-    <row r="861" spans="1:45" ht="15.75">
+    <row r="861" spans="1:45">
       <c r="A861" s="2">
         <v>4</v>
       </c>
@@ -60203,7 +60206,7 @@
       <c r="AR868" s="1"/>
       <c r="AS868" s="1"/>
     </row>
-    <row r="869" spans="1:45" ht="15.75">
+    <row r="869" spans="1:45">
       <c r="A869" s="2">
         <v>12</v>
       </c>
@@ -60633,7 +60636,7 @@
       <c r="AR876" s="1"/>
       <c r="AS876" s="1"/>
     </row>
-    <row r="877" spans="1:45" ht="15.75">
+    <row r="877" spans="1:45">
       <c r="A877" s="2">
         <v>17</v>
       </c>
@@ -61448,8 +61451,8 @@
       <c r="AC890" s="8" t="s">
         <v>1848</v>
       </c>
-      <c r="AD890" s="336"/>
-      <c r="AE890" s="337"/>
+      <c r="AD890" s="330"/>
+      <c r="AE890" s="328"/>
       <c r="AF890" s="1"/>
       <c r="AG890" s="2"/>
       <c r="AH890" s="1"/>
@@ -64450,7 +64453,7 @@
       <c r="AR945" s="1"/>
       <c r="AS945" s="1"/>
     </row>
-    <row r="946" spans="1:45" ht="15.75">
+    <row r="946" spans="1:45">
       <c r="A946" s="2">
         <v>11</v>
       </c>
@@ -64558,7 +64561,7 @@
       <c r="AR947" s="1"/>
       <c r="AS947" s="1"/>
     </row>
-    <row r="948" spans="1:45" ht="15.75">
+    <row r="948" spans="1:45">
       <c r="A948" s="2">
         <v>14</v>
       </c>
@@ -64660,7 +64663,7 @@
       <c r="AR949" s="1"/>
       <c r="AS949" s="1"/>
     </row>
-    <row r="950" spans="1:45" ht="15.75">
+    <row r="950" spans="1:45">
       <c r="A950" s="22" t="s">
         <v>27</v>
       </c>
@@ -64709,7 +64712,7 @@
       <c r="AR950" s="1"/>
       <c r="AS950" s="1"/>
     </row>
-    <row r="951" spans="1:45" ht="15.75">
+    <row r="951" spans="1:45">
       <c r="A951" s="22" t="s">
         <v>29</v>
       </c>
@@ -64758,7 +64761,7 @@
       <c r="AR951" s="1"/>
       <c r="AS951" s="1"/>
     </row>
-    <row r="952" spans="1:45" ht="15.75">
+    <row r="952" spans="1:45">
       <c r="A952" s="21" t="s">
         <v>31</v>
       </c>
@@ -64807,7 +64810,7 @@
       <c r="AR952" s="1"/>
       <c r="AS952" s="1"/>
     </row>
-    <row r="953" spans="1:45" ht="15.75">
+    <row r="953" spans="1:45">
       <c r="A953" s="2">
         <v>15</v>
       </c>
@@ -67453,7 +67456,7 @@
       <c r="AR1002" s="1"/>
       <c r="AS1002" s="1"/>
     </row>
-    <row r="1003" spans="1:45" ht="15.75">
+    <row r="1003" spans="1:45">
       <c r="A1003" s="2"/>
       <c r="B1003" s="2">
         <v>1</v>
@@ -67562,7 +67565,7 @@
       <c r="AR1003" s="1"/>
       <c r="AS1003" s="1"/>
     </row>
-    <row r="1004" spans="1:45" ht="15.75">
+    <row r="1004" spans="1:45">
       <c r="A1004" s="3" t="s">
         <v>0</v>
       </c>
@@ -67611,7 +67614,7 @@
       <c r="AR1004" s="1"/>
       <c r="AS1004" s="1"/>
     </row>
-    <row r="1005" spans="1:45" ht="15.75">
+    <row r="1005" spans="1:45">
       <c r="A1005" s="2">
         <v>1</v>
       </c>
@@ -67930,18 +67933,18 @@
       <c r="R1011" s="2"/>
       <c r="S1011" s="2"/>
       <c r="T1011" s="2"/>
-      <c r="U1011" s="336"/>
-      <c r="V1011" s="337"/>
-      <c r="W1011" s="337"/>
-      <c r="X1011" s="337"/>
-      <c r="Y1011" s="337"/>
-      <c r="Z1011" s="337"/>
-      <c r="AA1011" s="337"/>
-      <c r="AB1011" s="337"/>
-      <c r="AC1011" s="337"/>
-      <c r="AD1011" s="337"/>
-      <c r="AE1011" s="337"/>
-      <c r="AF1011" s="338"/>
+      <c r="U1011" s="330"/>
+      <c r="V1011" s="328"/>
+      <c r="W1011" s="328"/>
+      <c r="X1011" s="328"/>
+      <c r="Y1011" s="328"/>
+      <c r="Z1011" s="328"/>
+      <c r="AA1011" s="328"/>
+      <c r="AB1011" s="328"/>
+      <c r="AC1011" s="328"/>
+      <c r="AD1011" s="328"/>
+      <c r="AE1011" s="328"/>
+      <c r="AF1011" s="329"/>
       <c r="AG1011" s="2"/>
       <c r="AH1011" s="1"/>
       <c r="AI1011" s="1"/>
@@ -68554,7 +68557,7 @@
       <c r="AR1023" s="1"/>
       <c r="AS1023" s="1"/>
     </row>
-    <row r="1024" spans="1:45" ht="15.75">
+    <row r="1024" spans="1:45">
       <c r="A1024" s="2">
         <v>17</v>
       </c>
@@ -70115,7 +70118,7 @@
       <c r="AR1052" s="1"/>
       <c r="AS1052" s="1"/>
     </row>
-    <row r="1053" spans="1:45" ht="15.75">
+    <row r="1053" spans="1:45">
       <c r="A1053" s="2">
         <v>3</v>
       </c>
@@ -70166,7 +70169,7 @@
       <c r="AR1053" s="1"/>
       <c r="AS1053" s="1"/>
     </row>
-    <row r="1054" spans="1:45" ht="15.75">
+    <row r="1054" spans="1:45">
       <c r="A1054" s="2">
         <v>4</v>
       </c>
@@ -71695,7 +71698,7 @@
       <c r="AR1082" s="1"/>
       <c r="AS1082" s="1"/>
     </row>
-    <row r="1083" spans="1:45" ht="15.75">
+    <row r="1083" spans="1:45">
       <c r="A1083" s="2">
         <v>10</v>
       </c>
@@ -71746,7 +71749,7 @@
       <c r="AR1083" s="1"/>
       <c r="AS1083" s="1"/>
     </row>
-    <row r="1084" spans="1:45" ht="15.75">
+    <row r="1084" spans="1:45">
       <c r="A1084" s="2">
         <v>11</v>
       </c>
@@ -71797,7 +71800,7 @@
       <c r="AR1084" s="1"/>
       <c r="AS1084" s="1"/>
     </row>
-    <row r="1085" spans="1:45" ht="15.75">
+    <row r="1085" spans="1:45">
       <c r="A1085" s="2">
         <v>12</v>
       </c>
@@ -71899,7 +71902,7 @@
       <c r="AR1086" s="1"/>
       <c r="AS1086" s="1"/>
     </row>
-    <row r="1087" spans="1:45" ht="15.75">
+    <row r="1087" spans="1:45">
       <c r="A1087" s="21" t="s">
         <v>26</v>
       </c>
@@ -71997,7 +72000,7 @@
       <c r="AR1088" s="1"/>
       <c r="AS1088" s="1"/>
     </row>
-    <row r="1089" spans="1:45" ht="15.75">
+    <row r="1089" spans="1:45">
       <c r="A1089" s="22" t="s">
         <v>29</v>
       </c>
@@ -73222,7 +73225,7 @@
       <c r="AR1111" s="1"/>
       <c r="AS1111" s="1"/>
     </row>
-    <row r="1112" spans="1:45" ht="15.75">
+    <row r="1112" spans="1:45">
       <c r="A1112" s="22" t="s">
         <v>29</v>
       </c>
@@ -76644,7 +76647,7 @@
       <c r="AR1175" s="1"/>
       <c r="AS1175" s="1"/>
     </row>
-    <row r="1176" spans="1:45" ht="15.75">
+    <row r="1176" spans="1:45">
       <c r="A1176" s="2">
         <v>11</v>
       </c>
@@ -77138,20 +77141,54 @@
     </row>
   </sheetData>
   <mergeCells count="74">
-    <mergeCell ref="A1140:I1140"/>
-    <mergeCell ref="A1163:I1163"/>
-    <mergeCell ref="AE1011:AF1011"/>
-    <mergeCell ref="A1025:I1025"/>
-    <mergeCell ref="A1048:I1048"/>
-    <mergeCell ref="A1071:I1071"/>
-    <mergeCell ref="A1094:I1094"/>
-    <mergeCell ref="A1117:I1117"/>
-    <mergeCell ref="AC1011:AD1011"/>
-    <mergeCell ref="A1002:I1002"/>
-    <mergeCell ref="U1011:V1011"/>
-    <mergeCell ref="W1011:X1011"/>
-    <mergeCell ref="Y1011:Z1011"/>
-    <mergeCell ref="AA1011:AB1011"/>
+    <mergeCell ref="A109:I109"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A22:I22"/>
+    <mergeCell ref="A43:I43"/>
+    <mergeCell ref="A65:I65"/>
+    <mergeCell ref="A87:I87"/>
+    <mergeCell ref="A351:I351"/>
+    <mergeCell ref="G121:H121"/>
+    <mergeCell ref="A131:I131"/>
+    <mergeCell ref="A153:I153"/>
+    <mergeCell ref="A175:I175"/>
+    <mergeCell ref="A197:I197"/>
+    <mergeCell ref="A219:I219"/>
+    <mergeCell ref="A241:I241"/>
+    <mergeCell ref="A263:I263"/>
+    <mergeCell ref="A285:I285"/>
+    <mergeCell ref="A307:I307"/>
+    <mergeCell ref="A329:I329"/>
+    <mergeCell ref="AS352:AS353"/>
+    <mergeCell ref="AS355:AS356"/>
+    <mergeCell ref="AS358:AS361"/>
+    <mergeCell ref="AO360:AO361"/>
+    <mergeCell ref="AP360:AP361"/>
+    <mergeCell ref="AR360:AR361"/>
+    <mergeCell ref="A588:I588"/>
+    <mergeCell ref="A373:I373"/>
+    <mergeCell ref="A395:I395"/>
+    <mergeCell ref="A416:I416"/>
+    <mergeCell ref="A438:I438"/>
+    <mergeCell ref="A459:I459"/>
+    <mergeCell ref="A480:I480"/>
+    <mergeCell ref="A502:I502"/>
+    <mergeCell ref="A523:I523"/>
+    <mergeCell ref="A545:I545"/>
+    <mergeCell ref="F549:G549"/>
+    <mergeCell ref="A566:I566"/>
+    <mergeCell ref="A808:I808"/>
+    <mergeCell ref="A611:I611"/>
+    <mergeCell ref="A632:I632"/>
+    <mergeCell ref="A653:I653"/>
+    <mergeCell ref="A674:I674"/>
+    <mergeCell ref="A695:I695"/>
+    <mergeCell ref="A716:I716"/>
+    <mergeCell ref="A739:I739"/>
+    <mergeCell ref="A762:I762"/>
+    <mergeCell ref="F776:G776"/>
+    <mergeCell ref="H776:I776"/>
+    <mergeCell ref="A785:I785"/>
     <mergeCell ref="A979:I979"/>
     <mergeCell ref="W821:X821"/>
     <mergeCell ref="Y821:Z821"/>
@@ -77164,54 +77201,20 @@
     <mergeCell ref="A901:I901"/>
     <mergeCell ref="A933:I933"/>
     <mergeCell ref="A956:I956"/>
-    <mergeCell ref="A808:I808"/>
-    <mergeCell ref="A611:I611"/>
-    <mergeCell ref="A632:I632"/>
-    <mergeCell ref="A653:I653"/>
-    <mergeCell ref="A674:I674"/>
-    <mergeCell ref="A695:I695"/>
-    <mergeCell ref="A716:I716"/>
-    <mergeCell ref="A739:I739"/>
-    <mergeCell ref="A762:I762"/>
-    <mergeCell ref="F776:G776"/>
-    <mergeCell ref="H776:I776"/>
-    <mergeCell ref="A785:I785"/>
-    <mergeCell ref="A588:I588"/>
-    <mergeCell ref="A373:I373"/>
-    <mergeCell ref="A395:I395"/>
-    <mergeCell ref="A416:I416"/>
-    <mergeCell ref="A438:I438"/>
-    <mergeCell ref="A459:I459"/>
-    <mergeCell ref="A480:I480"/>
-    <mergeCell ref="A502:I502"/>
-    <mergeCell ref="A523:I523"/>
-    <mergeCell ref="A545:I545"/>
-    <mergeCell ref="F549:G549"/>
-    <mergeCell ref="A566:I566"/>
-    <mergeCell ref="AS352:AS353"/>
-    <mergeCell ref="AS355:AS356"/>
-    <mergeCell ref="AS358:AS361"/>
-    <mergeCell ref="AO360:AO361"/>
-    <mergeCell ref="AP360:AP361"/>
-    <mergeCell ref="AR360:AR361"/>
-    <mergeCell ref="A351:I351"/>
-    <mergeCell ref="G121:H121"/>
-    <mergeCell ref="A131:I131"/>
-    <mergeCell ref="A153:I153"/>
-    <mergeCell ref="A175:I175"/>
-    <mergeCell ref="A197:I197"/>
-    <mergeCell ref="A219:I219"/>
-    <mergeCell ref="A241:I241"/>
-    <mergeCell ref="A263:I263"/>
-    <mergeCell ref="A285:I285"/>
-    <mergeCell ref="A307:I307"/>
-    <mergeCell ref="A329:I329"/>
-    <mergeCell ref="A109:I109"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A22:I22"/>
-    <mergeCell ref="A43:I43"/>
-    <mergeCell ref="A65:I65"/>
-    <mergeCell ref="A87:I87"/>
+    <mergeCell ref="A1002:I1002"/>
+    <mergeCell ref="U1011:V1011"/>
+    <mergeCell ref="W1011:X1011"/>
+    <mergeCell ref="Y1011:Z1011"/>
+    <mergeCell ref="AA1011:AB1011"/>
+    <mergeCell ref="A1140:I1140"/>
+    <mergeCell ref="A1163:I1163"/>
+    <mergeCell ref="AE1011:AF1011"/>
+    <mergeCell ref="A1025:I1025"/>
+    <mergeCell ref="A1048:I1048"/>
+    <mergeCell ref="A1071:I1071"/>
+    <mergeCell ref="A1094:I1094"/>
+    <mergeCell ref="A1117:I1117"/>
+    <mergeCell ref="AC1011:AD1011"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>